<commit_message>
Module 1 workbooks updated with embedded practice sheets; link layout per workbook; module01b trims
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_cell_formatting.xlsx
+++ b/textbook_examples/mod01_cell_formatting.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_743D2901570355E50E650FA056691A6F79FBB9FE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3FE4A23-30BF-4645-8315-ACDDFF93987B}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="11_743D2901570355E50E650FA056691A6F79FBB9FE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35CBBE56-E98F-BF4E-9B29-39DEE7C257D5}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Formatting" sheetId="1" r:id="rId1"/>
+    <sheet name="Complete" sheetId="1" r:id="rId1"/>
+    <sheet name="Practice" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="31">
   <si>
     <t>To illustrate cell formatting on numbers let's take the number 0.5 and see the different ways it can be formatted</t>
   </si>
@@ -123,6 +124,9 @@
   </si>
   <si>
     <t>B12*2 (changed to general format)</t>
+  </si>
+  <si>
+    <t>In this worksheet all cells are formatted to general.  You can change the formatting to match the instructions Column A</t>
   </si>
 </sst>
 </file>
@@ -133,7 +137,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -200,6 +204,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -232,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -264,19 +274,25 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -597,22 +613,22 @@
       <c r="A2" s="1"/>
     </row>
     <row r="3" spans="1:4" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="18"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="20" t="s">
+      <c r="A3" s="15"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="18" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
     </row>
     <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
@@ -675,12 +691,12 @@
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
@@ -703,12 +719,12 @@
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
@@ -873,4 +889,303 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3EF9C7-25C6-E349-BD9A-9FE14EE7B2A4}">
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="34.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="13.5" customWidth="1"/>
+    <col min="4" max="4" width="62" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="23"/>
+      <c r="C3" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+    </row>
+    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="11">
+        <f>B5</f>
+        <v>0.5</v>
+      </c>
+      <c r="C6" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(B6)</f>
+        <v>=B5</v>
+      </c>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="11">
+        <f>B5</f>
+        <v>0.5</v>
+      </c>
+      <c r="C7" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(B7)</f>
+        <v>=B5</v>
+      </c>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="11">
+        <f>B5</f>
+        <v>0.5</v>
+      </c>
+      <c r="C8" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(B8)</f>
+        <v>=B5</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="5"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+    </row>
+    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="11">
+        <f>B6*2</f>
+        <v>1</v>
+      </c>
+      <c r="C11" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(B11)</f>
+        <v>=B6*2</v>
+      </c>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="5"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+    </row>
+    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="11">
+        <f>B6*2</f>
+        <v>1</v>
+      </c>
+      <c r="C14" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(B14)</f>
+        <v>=B6*2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="5"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="7"/>
+    </row>
+    <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="5"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="7"/>
+    </row>
+    <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="11">
+        <v>2.4</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="11">
+        <v>2.4</v>
+      </c>
+      <c r="C19" s="7"/>
+      <c r="D19" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" s="11">
+        <f>B18+B19</f>
+        <v>4.8</v>
+      </c>
+      <c r="C20" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(B20)</f>
+        <v>=B18+B19</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="5"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" s="19">
+        <v>46272</v>
+      </c>
+      <c r="C24" s="7"/>
+      <c r="D24" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="11">
+        <f>B24</f>
+        <v>46272</v>
+      </c>
+      <c r="C25" s="7"/>
+      <c r="D25" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="11">
+        <f>B24+7</f>
+        <v>46279</v>
+      </c>
+      <c r="C26" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(B26)</f>
+        <v>=B24+7</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="7"/>
+      <c r="D27" s="2"/>
+    </row>
+    <row r="28" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="11" t="e">
+        <f>B27+7</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C28" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(B28)</f>
+        <v>=B27+7</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add sorting-and-filtering workbook to module01b; commit latest workbook saves
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_cell_formatting.xlsx
+++ b/textbook_examples/mod01_cell_formatting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="11_743D2901570355E50E650FA056691A6F79FBB9FE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35CBBE56-E98F-BF4E-9B29-39DEE7C257D5}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="11_743D2901570355E50E650FA056691A6F79FBB9FE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A424A728-F23B-334E-AD20-83CFC078F997}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -242,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -292,6 +292,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -944,7 +947,7 @@
       <c r="A6" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="24">
         <f>B5</f>
         <v>0.5</v>
       </c>
@@ -958,7 +961,7 @@
       <c r="A7" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="24">
         <f>B5</f>
         <v>0.5</v>
       </c>
@@ -972,7 +975,7 @@
       <c r="A8" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="24">
         <f>B5</f>
         <v>0.5</v>
       </c>
@@ -1000,14 +1003,8 @@
       <c r="A11" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="11">
-        <f>B6*2</f>
-        <v>1</v>
-      </c>
-      <c r="C11" s="7" t="str">
-        <f ca="1">_xlfn.FORMULATEXT(B11)</f>
-        <v>=B6*2</v>
-      </c>
+      <c r="B11" s="24"/>
+      <c r="C11" s="7"/>
       <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1059,7 +1056,7 @@
       <c r="A18" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="24">
         <v>2.4</v>
       </c>
       <c r="C18" s="7"/>
@@ -1071,7 +1068,7 @@
       <c r="A19" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="24">
         <v>2.4</v>
       </c>
       <c r="C19" s="7"/>
@@ -1083,7 +1080,7 @@
       <c r="A20" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="24">
         <f>B18+B19</f>
         <v>4.8</v>
       </c>
@@ -1126,7 +1123,7 @@
       <c r="A25" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="14">
         <f>B24</f>
         <v>46272</v>
       </c>
@@ -1139,13 +1136,10 @@
       <c r="A26" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="11">
-        <f>B24+7</f>
-        <v>46279</v>
-      </c>
-      <c r="C26" s="7" t="str">
+      <c r="B26" s="24"/>
+      <c r="C26" s="7" t="e">
         <f ca="1">_xlfn.FORMULATEXT(B26)</f>
-        <v>=B24+7</v>
+        <v>#N/A</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>18</v>
@@ -1165,13 +1159,10 @@
       <c r="A28" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="11" t="e">
-        <f>B27+7</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C28" s="7" t="str">
+      <c r="B28" s="11"/>
+      <c r="C28" s="7" t="e">
         <f ca="1">_xlfn.FORMULATEXT(B28)</f>
-        <v>=B27+7</v>
+        <v>#N/A</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>21</v>

</xml_diff>